<commit_message>
fix(excel): repair desktop workbook open
</commit_message>
<xml_diff>
--- a/Python/structural_lib/data/excel/outputs/e1-excel-routine-workbench/structural-lib-rectangular-beam-workbench-v1.xlsx
+++ b/Python/structural_lib/data/excel/outputs/e1-excel-routine-workbench/structural-lib-rectangular-beam-workbench-v1.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workbook_Info" sheetId="1" r:id="Rd75f3e9e45314595"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Beam_Workbench" sheetId="2" r:id="R99d72ec1d70a43f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mapping_Preview" sheetId="3" r:id="Re470ac26aebf4535"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Row_Ledger" sheetId="4" r:id="Rce13deb30e6940aa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Results" sheetId="5" r:id="R1258e99719474668"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Passports" sheetId="6" r:id="Raf883d501e034ddb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workbook_Info" sheetId="1" r:id="rId4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Beam_Workbench" sheetId="2" r:id="rId5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mapping_Preview" sheetId="3" r:id="rId6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Row_Ledger" sheetId="4" r:id="rId7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Results" sheetId="5" r:id="rId8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Passports" sheetId="6" r:id="rId9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -21,7 +21,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="200" formatCode="0.00"/>
   </x:numFmts>
-  <x:fonts count="5">
+  <x:fonts count="7">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -45,13 +45,23 @@
       <x:name val="Carlito"/>
     </x:font>
     <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF137333"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF9A6700"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
       <x:b/>
       <x:sz val="11"/>
       <x:color rgb="FF9A6700"/>
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="9">
+  <x:fills count="8">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -80,12 +90,7 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFFFFFF"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFFF4CE"/>
+        <x:fgColor rgb="FFE6F4EA"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -94,34 +99,12 @@
       </x:patternFill>
     </x:fill>
   </x:fills>
-  <x:borders count="16">
+  <x:borders count="13">
     <x:border/>
     <x:border>
       <x:left style="thin">
         <x:color rgb="FFC8D2DA"/>
       </x:left>
-      <x:right style="thin">
-        <x:color rgb="FFC8D2DA"/>
-      </x:right>
-      <x:top style="thin">
-        <x:color rgb="FFC8D2DA"/>
-      </x:top>
-      <x:bottom style="thin">
-        <x:color rgb="FFC8D2DA"/>
-      </x:bottom>
-    </x:border>
-    <x:border>
-      <x:left style="thin">
-        <x:color rgb="FFC8D2DA"/>
-      </x:left>
-      <x:top style="thin">
-        <x:color rgb="FFC8D2DA"/>
-      </x:top>
-      <x:bottom style="thin">
-        <x:color rgb="FFC8D2DA"/>
-      </x:bottom>
-    </x:border>
-    <x:border>
       <x:right style="thin">
         <x:color rgb="FFC8D2DA"/>
       </x:right>
@@ -178,14 +161,6 @@
       <x:top style="thin">
         <x:color rgb="FFC8D2DA"/>
       </x:top>
-      <x:bottom style="thin">
-        <x:color rgb="FFC8D2DA"/>
-      </x:bottom>
-    </x:border>
-    <x:border>
-      <x:top style="thin">
-        <x:color rgb="FFC8D2DA"/>
-      </x:top>
     </x:border>
     <x:border>
       <x:bottom style="thin">
@@ -226,249 +201,97 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="71">
+  <x:cellXfs count="52">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="200" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="7" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="7" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="7" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="7" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="7" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="7" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="8">
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF137333"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFE6F4EA"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF9A6700"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFFF4CE"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF9A6700"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFFF4CE"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF137333"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFE6F4EA"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FFB3261E"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFCE8E6"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FFB3261E"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFCE8E6"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF137333"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFE6F4EA"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FFB3261E"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFCE8E6"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-  </x:dxfs>
 </x:styleSheet>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tbl_Beam_Workbench_V1" displayName="tbl_Beam_Workbench_V1" ref="A4:Q7" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:Q7"/>
   <x:tableColumns count="17">
     <x:tableColumn id="1" name="Row ID"/>
     <x:tableColumn id="2" name="Beam ID"/>
@@ -478,7 +301,7 @@
     <x:tableColumn id="6" name="b (mm)"/>
     <x:tableColumn id="7" name="D (mm)"/>
     <x:tableColumn id="8" name="Depth Basis"/>
-    <x:tableColumn id="9" name="d (mm)"/>
+    <x:tableColumn id="9" name="Effective d (mm)"/>
     <x:tableColumn id="10" name="Clear Cover (mm)"/>
     <x:tableColumn id="11" name="Stirrup Dia (mm)"/>
     <x:tableColumn id="12" name="Tension Bar Dia (mm)"/>
@@ -494,6 +317,7 @@
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tbl_Mapping_Preview_V1" displayName="tbl_Mapping_Preview_V1" ref="A4:D21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:D21"/>
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Canonical Field"/>
     <x:tableColumn id="2" name="Source Header"/>
@@ -506,6 +330,7 @@
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="tbl_Row_Ledger_V1" displayName="tbl_Row_Ledger_V1" ref="A4:I5" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:I5"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Source Row"/>
     <x:tableColumn id="2" name="Row ID"/>
@@ -523,6 +348,7 @@
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="tbl_Results_V1" displayName="tbl_Results_V1" ref="A4:J5" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:J5"/>
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="Row ID"/>
     <x:tableColumn id="2" name="Beam ID"/>
@@ -541,6 +367,7 @@
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="tbl_Passports_V1" displayName="tbl_Passports_V1" ref="A4:L5" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:L5"/>
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="Row ID"/>
     <x:tableColumn id="2" name="Beam ID"/>
@@ -754,211 +581,224 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="25" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="42" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="26" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="44" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="4" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="20" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="34" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="44" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="30" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="40" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="56" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
-      <x:c r="A1" s="3" t="str">
+      <x:c r="A1" s="2" t="str">
         <x:v>Excel Routine Workbench V1</x:v>
       </x:c>
+      <x:c r="B1" s="2"/>
+      <x:c r="C1" s="2"/>
+      <x:c r="D1" s="2"/>
+      <x:c r="E1" s="2"/>
+      <x:c r="F1" s="2"/>
     </x:row>
     <x:row r="2" ht="30" customHeight="1">
-      <x:c r="A2" s="8" t="str">
+      <x:c r="A2" s="6" t="str">
         <x:v>Macro-free Office.js workbook. Structural calculations run only through structural_lib design_beam_is456; this file contains no structural-design formulas.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="4" ht="30" customHeight="1">
-      <x:c r="A4" s="15" t="str">
+      <x:c r="B2" s="6"/>
+      <x:c r="C2" s="6"/>
+      <x:c r="D2" s="6"/>
+      <x:c r="E2" s="6"/>
+      <x:c r="F2" s="6"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="10" t="str">
         <x:v>Workbook identity</x:v>
       </x:c>
-      <x:c r="B4" s="16" t="str">
+      <x:c r="B4" s="10" t="str">
         <x:v>Value</x:v>
       </x:c>
-      <x:c r="D4" s="15" t="str">
+      <x:c r="D4" s="10" t="str">
         <x:v>Capability</x:v>
       </x:c>
-      <x:c r="E4" s="32" t="str">
+      <x:c r="E4" s="10" t="str">
         <x:v>State</x:v>
       </x:c>
-      <x:c r="F4" s="16" t="str">
+      <x:c r="F4" s="10" t="str">
         <x:v>Meaning</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="24" t="str">
+      <x:c r="A5" s="12" t="str">
         <x:v>Template ID</x:v>
       </x:c>
-      <x:c r="B5" s="25" t="str">
+      <x:c r="B5" s="13" t="str">
         <x:v>structural-lib-rectangular-beam-workbench</x:v>
       </x:c>
-      <x:c r="D5" s="42" t="str">
+      <x:c r="D5" s="18" t="str">
         <x:v>E1 software</x:v>
       </x:c>
-      <x:c r="E5" s="43" t="str">
+      <x:c r="E5" s="37" t="str">
         <x:v>AVAILABLE</x:v>
       </x:c>
-      <x:c r="F5" s="44" t="str">
+      <x:c r="F5" s="20" t="str">
         <x:v>Contract, API, workbook, and task pane implemented</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="26" t="str">
+      <x:c r="A6" s="14" t="str">
         <x:v>Template version</x:v>
       </x:c>
-      <x:c r="B6" s="27" t="str">
+      <x:c r="B6" s="15" t="str">
         <x:v>1.0</x:v>
       </x:c>
-      <x:c r="D6" s="45" t="str">
+      <x:c r="D6" s="21" t="str">
         <x:v>Windows Excel runtime</x:v>
       </x:c>
-      <x:c r="E6" s="46" t="str">
+      <x:c r="E6" s="40" t="str">
         <x:v>TO_VERIFY_WINDOWS</x:v>
       </x:c>
-      <x:c r="F6" s="47" t="str">
+      <x:c r="F6" s="23" t="str">
         <x:v>Requires the separate installed-Windows evidence gate</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="26" t="str">
+      <x:c r="A7" s="14" t="str">
         <x:v>Contract schema</x:v>
       </x:c>
-      <x:c r="B7" s="27" t="str">
+      <x:c r="B7" s="15" t="str">
         <x:v>excel-workbook-contract/v1</x:v>
       </x:c>
-      <x:c r="D7" s="48" t="str">
+      <x:c r="D7" s="24" t="str">
         <x:v>Qualified engineering review</x:v>
       </x:c>
-      <x:c r="E7" s="49" t="str">
+      <x:c r="E7" s="41" t="str">
         <x:v>REQUIRED</x:v>
       </x:c>
-      <x:c r="F7" s="50" t="str">
+      <x:c r="F7" s="26" t="str">
         <x:v>Software output is not professional approval</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="26" t="str">
+      <x:c r="A8" s="14" t="str">
         <x:v>Input worksheet</x:v>
       </x:c>
-      <x:c r="B8" s="27" t="str">
+      <x:c r="B8" s="15" t="str">
         <x:v>Beam_Workbench</x:v>
       </x:c>
-    </x:row>
-    <x:row r="9" ht="30" customHeight="1">
-      <x:c r="A9" s="26" t="str">
+      <x:c r="D8"/>
+      <x:c r="E8"/>
+      <x:c r="F8"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="14" t="str">
         <x:v>Input table</x:v>
       </x:c>
-      <x:c r="B9" s="27" t="str">
+      <x:c r="B9" s="15" t="str">
         <x:v>tbl_Beam_Workbench_V1</x:v>
       </x:c>
-      <x:c r="D9" s="15" t="str">
+      <x:c r="D9" s="10" t="str">
         <x:v>Workflow</x:v>
       </x:c>
-      <x:c r="E9" s="32" t="str">
+      <x:c r="E9" s="10" t="str">
         <x:v>Rule</x:v>
       </x:c>
-      <x:c r="F9" s="16" t="str">
+      <x:c r="F9" s="10" t="str">
         <x:v>Why it matters</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="28" customHeight="1">
-      <x:c r="A10" s="26" t="str">
+    <x:row r="10">
+      <x:c r="A10" s="14" t="str">
         <x:v>Unit system</x:v>
       </x:c>
-      <x:c r="B10" s="27" t="str">
+      <x:c r="B10" s="15" t="str">
         <x:v>IS456</x:v>
       </x:c>
-      <x:c r="D10" s="51" t="str">
+      <x:c r="D10" s="27" t="str">
         <x:v>1. Select</x:v>
       </x:c>
-      <x:c r="E10" s="52" t="str">
+      <x:c r="E10" s="28" t="str">
         <x:v>Use only tbl_Beam_Workbench_V1</x:v>
       </x:c>
-      <x:c r="F10" s="53" t="str">
+      <x:c r="F10" s="29" t="str">
         <x:v>Binds worksheet and table identity</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="28" customHeight="1">
-      <x:c r="A11" s="26" t="str">
+    <x:row r="11">
+      <x:c r="A11" s="14" t="str">
         <x:v>Trust mode</x:v>
       </x:c>
-      <x:c r="B11" s="27" t="str">
+      <x:c r="B11" s="15" t="str">
         <x:v>MACRO_FREE_OFFICE_JS</x:v>
       </x:c>
-      <x:c r="D11" s="54" t="str">
+      <x:c r="D11" s="30" t="str">
         <x:v>2. Preview</x:v>
       </x:c>
-      <x:c r="E11" s="55" t="str">
+      <x:c r="E11" s="31" t="str">
         <x:v>Review the exact header mapping</x:v>
       </x:c>
-      <x:c r="F11" s="56" t="str">
+      <x:c r="F11" s="32" t="str">
         <x:v>Blocks missing or duplicate mappings</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="28" customHeight="1">
-      <x:c r="A12" s="26" t="str">
+    <x:row r="12">
+      <x:c r="A12" s="14" t="str">
         <x:v>Torsion scope</x:v>
       </x:c>
-      <x:c r="B12" s="27" t="str">
+      <x:c r="B12" s="15" t="str">
         <x:v>DISABLED_E1</x:v>
       </x:c>
-      <x:c r="D12" s="54" t="str">
+      <x:c r="D12" s="30" t="str">
         <x:v>3. Run</x:v>
       </x:c>
-      <x:c r="E12" s="55" t="str">
+      <x:c r="E12" s="31" t="str">
         <x:v>Confirm the mapping hash</x:v>
       </x:c>
-      <x:c r="F12" s="56" t="str">
+      <x:c r="F12" s="32" t="str">
         <x:v>Prevents unreviewed remapping</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="28" customHeight="1">
-      <x:c r="A13" s="26" t="str">
+    <x:row r="13">
+      <x:c r="A13" s="14" t="str">
         <x:v>Serviceability scope</x:v>
       </x:c>
-      <x:c r="B13" s="27" t="str">
+      <x:c r="B13" s="15" t="str">
         <x:v>DISABLED_E1</x:v>
       </x:c>
-      <x:c r="D13" s="54" t="str">
+      <x:c r="D13" s="30" t="str">
         <x:v>4. Review</x:v>
       </x:c>
-      <x:c r="E13" s="55" t="str">
+      <x:c r="E13" s="31" t="str">
         <x:v>Inspect ledger, results, passports</x:v>
       </x:c>
-      <x:c r="F13" s="56" t="str">
+      <x:c r="F13" s="32" t="str">
         <x:v>Every source row is accounted for</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="28" customHeight="1">
-      <x:c r="A14" s="28" t="str">
+    <x:row r="14">
+      <x:c r="A14" s="16" t="str">
         <x:v>Canonical function</x:v>
       </x:c>
-      <x:c r="B14" s="29" t="str">
+      <x:c r="B14" s="17" t="str">
         <x:v>design_beam_is456</x:v>
       </x:c>
-      <x:c r="D14" s="57" t="str">
+      <x:c r="D14" s="33" t="str">
         <x:v>5. Recheck</x:v>
       </x:c>
-      <x:c r="E14" s="58" t="str">
+      <x:c r="E14" s="34" t="str">
         <x:v>Treat edits as stale immediately</x:v>
       </x:c>
-      <x:c r="F14" s="59" t="str">
+      <x:c r="F14" s="35" t="str">
         <x:v>Prevents reuse of superseded output</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="34" customHeight="1">
-      <x:c r="A16" s="65" t="str">
+    <x:row r="16" ht="30" customHeight="1">
+      <x:c r="A16" s="46" t="str">
         <x:v>Held in E1: torsion, serviceability, ETABS import/write-back, hidden defaults, VBA/macros, and release or qualified-approval claims.</x:v>
       </x:c>
-      <x:c r="B16" s="66"/>
-      <x:c r="C16" s="66"/>
-      <x:c r="D16" s="66"/>
-      <x:c r="E16" s="66"/>
-      <x:c r="F16" s="67"/>
+      <x:c r="B16" s="47"/>
+      <x:c r="C16" s="47"/>
+      <x:c r="D16" s="47"/>
+      <x:c r="E16" s="47"/>
+      <x:c r="F16" s="48"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -966,11 +806,6 @@
     <x:mergeCell ref="A2:F2"/>
     <x:mergeCell ref="A16:F16"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="E5:E7">
-    <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="AVAILABLE"/>
-    <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="TO_VERIFY"/>
-    <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="REQUIRED"/>
-  </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
@@ -987,10 +822,10 @@
     <x:col min="6" max="6" width="14" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="22" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="17" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="20" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="17" hidden="0" customWidth="1"/>
     <x:col min="11" max="11" width="17" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="17" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="20" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="17" hidden="0" customWidth="1"/>
     <x:col min="14" max="14" width="17" hidden="0" customWidth="1"/>
     <x:col min="15" max="15" width="17" hidden="0" customWidth="1"/>
@@ -999,14 +834,46 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
-      <x:c r="A1" s="3" t="str">
+      <x:c r="A1" s="2" t="str">
         <x:v>Rectangular Beam Input Workbench — IS 456</x:v>
       </x:c>
+      <x:c r="B1" s="2"/>
+      <x:c r="C1" s="2"/>
+      <x:c r="D1" s="2"/>
+      <x:c r="E1" s="2"/>
+      <x:c r="F1" s="2"/>
+      <x:c r="G1" s="2"/>
+      <x:c r="H1" s="2"/>
+      <x:c r="I1" s="2"/>
+      <x:c r="J1" s="2"/>
+      <x:c r="K1" s="2"/>
+      <x:c r="L1" s="2"/>
+      <x:c r="M1" s="2"/>
+      <x:c r="N1" s="2"/>
+      <x:c r="O1" s="2"/>
+      <x:c r="P1" s="2"/>
+      <x:c r="Q1" s="2"/>
     </x:row>
     <x:row r="2" ht="30" customHeight="1">
-      <x:c r="A2" s="8" t="str">
+      <x:c r="A2" s="6" t="str">
         <x:v>Yellow cells are user inputs. Numeric text such as '300' is blocked; enter actual numbers. Blank table rows are retained as EXCLUDED in the row ledger.</x:v>
       </x:c>
+      <x:c r="B2" s="6"/>
+      <x:c r="C2" s="6"/>
+      <x:c r="D2" s="6"/>
+      <x:c r="E2" s="6"/>
+      <x:c r="F2" s="6"/>
+      <x:c r="G2" s="6"/>
+      <x:c r="H2" s="6"/>
+      <x:c r="I2" s="6"/>
+      <x:c r="J2" s="6"/>
+      <x:c r="K2" s="6"/>
+      <x:c r="L2" s="6"/>
+      <x:c r="M2" s="6"/>
+      <x:c r="N2" s="6"/>
+      <x:c r="O2" s="6"/>
+      <x:c r="P2" s="6"/>
+      <x:c r="Q2" s="6"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="str">
@@ -1034,7 +901,7 @@
         <x:v>Depth Basis</x:v>
       </x:c>
       <x:c r="I4" t="str">
-        <x:v>d (mm)</x:v>
+        <x:v>Effective d (mm)</x:v>
       </x:c>
       <x:c r="J4" t="str">
         <x:v>Clear Cover (mm)</x:v>
@@ -1062,121 +929,121 @@
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="68" t="str">
+      <x:c r="A5" s="38" t="str">
         <x:v>R1</x:v>
       </x:c>
-      <x:c r="B5" s="68" t="str">
+      <x:c r="B5" s="38" t="str">
         <x:v>B1</x:v>
       </x:c>
-      <x:c r="C5" s="68" t="str">
+      <x:c r="C5" s="38" t="str">
         <x:v>ULS-1</x:v>
       </x:c>
-      <x:c r="D5" s="69" t="n">
+      <x:c r="D5" s="49" t="n">
         <x:v>150</x:v>
       </x:c>
-      <x:c r="E5" s="69" t="n">
+      <x:c r="E5" s="49" t="n">
         <x:v>100</x:v>
       </x:c>
-      <x:c r="F5" s="69" t="n">
+      <x:c r="F5" s="49" t="n">
         <x:v>300</x:v>
       </x:c>
-      <x:c r="G5" s="69" t="n">
+      <x:c r="G5" s="49" t="n">
         <x:v>500</x:v>
       </x:c>
-      <x:c r="H5" s="68" t="str">
+      <x:c r="H5" s="38" t="str">
         <x:v>DERIVED_FROM_BARS</x:v>
       </x:c>
-      <x:c r="I5" s="69"/>
-      <x:c r="J5" s="69" t="n">
+      <x:c r="I5" s="49"/>
+      <x:c r="J5" s="49" t="n">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="K5" s="69" t="n">
+      <x:c r="K5" s="49" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="L5" s="69" t="n">
+      <x:c r="L5" s="49" t="n">
         <x:v>18</x:v>
       </x:c>
-      <x:c r="M5" s="69"/>
-      <x:c r="N5" s="69" t="n">
+      <x:c r="M5" s="49"/>
+      <x:c r="N5" s="49" t="n">
         <x:v>100</x:v>
       </x:c>
-      <x:c r="O5" s="69" t="n">
+      <x:c r="O5" s="49" t="n">
         <x:v>25</x:v>
       </x:c>
-      <x:c r="P5" s="69" t="n">
+      <x:c r="P5" s="49" t="n">
         <x:v>500</x:v>
       </x:c>
-      <x:c r="Q5" s="68" t="str">
+      <x:c r="Q5" s="38" t="str">
         <x:v>AUTO_FROM_FLEXURE</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="68" t="str">
+      <x:c r="A6" s="38" t="str">
         <x:v>R2</x:v>
       </x:c>
-      <x:c r="B6" s="68" t="str">
+      <x:c r="B6" s="38" t="str">
         <x:v>B2</x:v>
       </x:c>
-      <x:c r="C6" s="68" t="str">
+      <x:c r="C6" s="38" t="str">
         <x:v>ULS-2</x:v>
       </x:c>
-      <x:c r="D6" s="69" t="n">
+      <x:c r="D6" s="49" t="n">
         <x:v>150</x:v>
       </x:c>
-      <x:c r="E6" s="69" t="n">
+      <x:c r="E6" s="49" t="n">
         <x:v>420</x:v>
       </x:c>
-      <x:c r="F6" s="69" t="n">
+      <x:c r="F6" s="49" t="n">
         <x:v>300</x:v>
       </x:c>
-      <x:c r="G6" s="69" t="n">
+      <x:c r="G6" s="49" t="n">
         <x:v>500</x:v>
       </x:c>
-      <x:c r="H6" s="68" t="str">
+      <x:c r="H6" s="38" t="str">
         <x:v>EXPLICIT_D</x:v>
       </x:c>
-      <x:c r="I6" s="69" t="n">
+      <x:c r="I6" s="49" t="n">
         <x:v>443</x:v>
       </x:c>
-      <x:c r="J6" s="69"/>
-      <x:c r="K6" s="69" t="n">
+      <x:c r="J6" s="49"/>
+      <x:c r="K6" s="49" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="L6" s="69"/>
-      <x:c r="M6" s="69" t="n">
+      <x:c r="L6" s="49"/>
+      <x:c r="M6" s="49" t="n">
         <x:v>57</x:v>
       </x:c>
-      <x:c r="N6" s="69" t="n">
+      <x:c r="N6" s="49" t="n">
         <x:v>100</x:v>
       </x:c>
-      <x:c r="O6" s="69" t="n">
+      <x:c r="O6" s="49" t="n">
         <x:v>25</x:v>
       </x:c>
-      <x:c r="P6" s="69" t="n">
+      <x:c r="P6" s="49" t="n">
         <x:v>500</x:v>
       </x:c>
-      <x:c r="Q6" s="68" t="str">
+      <x:c r="Q6" s="38" t="str">
         <x:v>AUTO_FROM_FLEXURE</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="68"/>
-      <x:c r="B7" s="68"/>
-      <x:c r="C7" s="68"/>
-      <x:c r="D7" s="69"/>
-      <x:c r="E7" s="69"/>
-      <x:c r="F7" s="69"/>
-      <x:c r="G7" s="69"/>
-      <x:c r="H7" s="68"/>
-      <x:c r="I7" s="69"/>
-      <x:c r="J7" s="69"/>
-      <x:c r="K7" s="69"/>
-      <x:c r="L7" s="69"/>
-      <x:c r="M7" s="69"/>
-      <x:c r="N7" s="69"/>
-      <x:c r="O7" s="69"/>
-      <x:c r="P7" s="69"/>
-      <x:c r="Q7" s="68"/>
+      <x:c r="A7" s="38"/>
+      <x:c r="B7" s="38"/>
+      <x:c r="C7" s="38"/>
+      <x:c r="D7" s="49"/>
+      <x:c r="E7" s="49"/>
+      <x:c r="F7" s="49"/>
+      <x:c r="G7" s="49"/>
+      <x:c r="H7" s="38"/>
+      <x:c r="I7" s="49"/>
+      <x:c r="J7" s="49"/>
+      <x:c r="K7" s="49"/>
+      <x:c r="L7" s="49"/>
+      <x:c r="M7" s="49"/>
+      <x:c r="N7" s="49"/>
+      <x:c r="O7" s="49"/>
+      <x:c r="P7" s="49"/>
+      <x:c r="Q7" s="38"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1193,7 +1060,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb591b26fc1b94de5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1202,21 +1069,27 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="28" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="27" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="15" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="40" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="26" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="38" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
-      <x:c r="A1" s="3" t="str">
+      <x:c r="A1" s="2" t="str">
         <x:v>Mapping Preview</x:v>
       </x:c>
+      <x:c r="B1" s="2"/>
+      <x:c r="C1" s="2"/>
+      <x:c r="D1" s="2"/>
     </x:row>
     <x:row r="2" ht="30" customHeight="1">
-      <x:c r="A2" s="8" t="str">
+      <x:c r="A2" s="6" t="str">
         <x:v>Review these mappings in the task pane before Run. A changed mapping invalidates the prior confirmation hash.</x:v>
       </x:c>
+      <x:c r="B2" s="6"/>
+      <x:c r="C2" s="6"/>
+      <x:c r="D2" s="6"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="str">
@@ -1239,7 +1112,7 @@
       <x:c r="B5" t="str">
         <x:v>Row ID</x:v>
       </x:c>
-      <x:c r="C5" t="str">
+      <x:c r="C5" s="51" t="str">
         <x:v>READY</x:v>
       </x:c>
       <x:c r="D5" t="str">
@@ -1253,7 +1126,7 @@
       <x:c r="B6" t="str">
         <x:v>Beam ID</x:v>
       </x:c>
-      <x:c r="C6" t="str">
+      <x:c r="C6" s="51" t="str">
         <x:v>READY</x:v>
       </x:c>
       <x:c r="D6" t="str">
@@ -1267,7 +1140,7 @@
       <x:c r="B7" t="str">
         <x:v>Case ID</x:v>
       </x:c>
-      <x:c r="C7" t="str">
+      <x:c r="C7" s="51" t="str">
         <x:v>READY</x:v>
       </x:c>
       <x:c r="D7" t="str">
@@ -1281,7 +1154,7 @@
       <x:c r="B8" t="str">
         <x:v>Mu (kN·m)</x:v>
       </x:c>
-      <x:c r="C8" t="str">
+      <x:c r="C8" s="51" t="str">
         <x:v>READY</x:v>
       </x:c>
       <x:c r="D8" t="str">
@@ -1295,7 +1168,7 @@
       <x:c r="B9" t="str">
         <x:v>Vu (kN)</x:v>
       </x:c>
-      <x:c r="C9" t="str">
+      <x:c r="C9" s="51" t="str">
         <x:v>READY</x:v>
       </x:c>
       <x:c r="D9" t="str">
@@ -1309,7 +1182,7 @@
       <x:c r="B10" t="str">
         <x:v>b (mm)</x:v>
       </x:c>
-      <x:c r="C10" t="str">
+      <x:c r="C10" s="51" t="str">
         <x:v>READY</x:v>
       </x:c>
       <x:c r="D10" t="str">
@@ -1323,7 +1196,7 @@
       <x:c r="B11" t="str">
         <x:v>D (mm)</x:v>
       </x:c>
-      <x:c r="C11" t="str">
+      <x:c r="C11" s="51" t="str">
         <x:v>READY</x:v>
       </x:c>
       <x:c r="D11" t="str">
@@ -1337,7 +1210,7 @@
       <x:c r="B12" t="str">
         <x:v>Depth Basis</x:v>
       </x:c>
-      <x:c r="C12" t="str">
+      <x:c r="C12" s="51" t="str">
         <x:v>READY</x:v>
       </x:c>
       <x:c r="D12" t="str">
@@ -1349,9 +1222,9 @@
         <x:v>d_mm</x:v>
       </x:c>
       <x:c r="B13" t="str">
-        <x:v>d (mm)</x:v>
-      </x:c>
-      <x:c r="C13" t="str">
+        <x:v>Effective d (mm)</x:v>
+      </x:c>
+      <x:c r="C13" s="51" t="str">
         <x:v>READY</x:v>
       </x:c>
       <x:c r="D13" t="str">
@@ -1365,7 +1238,7 @@
       <x:c r="B14" t="str">
         <x:v>Clear Cover (mm)</x:v>
       </x:c>
-      <x:c r="C14" t="str">
+      <x:c r="C14" s="51" t="str">
         <x:v>READY</x:v>
       </x:c>
       <x:c r="D14" t="str">
@@ -1379,7 +1252,7 @@
       <x:c r="B15" t="str">
         <x:v>Stirrup Dia (mm)</x:v>
       </x:c>
-      <x:c r="C15" t="str">
+      <x:c r="C15" s="51" t="str">
         <x:v>READY</x:v>
       </x:c>
       <x:c r="D15" t="str">
@@ -1393,7 +1266,7 @@
       <x:c r="B16" t="str">
         <x:v>Tension Bar Dia (mm)</x:v>
       </x:c>
-      <x:c r="C16" t="str">
+      <x:c r="C16" s="51" t="str">
         <x:v>READY</x:v>
       </x:c>
       <x:c r="D16" t="str">
@@ -1407,7 +1280,7 @@
       <x:c r="B17" t="str">
         <x:v>d' (mm)</x:v>
       </x:c>
-      <x:c r="C17" t="str">
+      <x:c r="C17" s="51" t="str">
         <x:v>READY</x:v>
       </x:c>
       <x:c r="D17" t="str">
@@ -1421,7 +1294,7 @@
       <x:c r="B18" t="str">
         <x:v>Asv (mm²)</x:v>
       </x:c>
-      <x:c r="C18" t="str">
+      <x:c r="C18" s="51" t="str">
         <x:v>READY</x:v>
       </x:c>
       <x:c r="D18" t="str">
@@ -1435,7 +1308,7 @@
       <x:c r="B19" t="str">
         <x:v>fck (N/mm²)</x:v>
       </x:c>
-      <x:c r="C19" t="str">
+      <x:c r="C19" s="51" t="str">
         <x:v>READY</x:v>
       </x:c>
       <x:c r="D19" t="str">
@@ -1449,7 +1322,7 @@
       <x:c r="B20" t="str">
         <x:v>fy (N/mm²)</x:v>
       </x:c>
-      <x:c r="C20" t="str">
+      <x:c r="C20" s="51" t="str">
         <x:v>READY</x:v>
       </x:c>
       <x:c r="D20" t="str">
@@ -1463,7 +1336,7 @@
       <x:c r="B21" t="str">
         <x:v>Shear Basis</x:v>
       </x:c>
-      <x:c r="C21" t="str">
+      <x:c r="C21" s="51" t="str">
         <x:v>READY</x:v>
       </x:c>
       <x:c r="D21" t="str">
@@ -1475,13 +1348,9 @@
     <x:mergeCell ref="A1:D1"/>
     <x:mergeCell ref="A2:D2"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="C5:C204">
-    <x:cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="READY"/>
-    <x:cfRule type="containsText" dxfId="4" priority="2" operator="containsText" text="BLOCKED"/>
-  </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6735982669f447d6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1490,26 +1359,42 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="13" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="20" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="20" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="20" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="23" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="23" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="23" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="22" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="36" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="36" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="36" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
-      <x:c r="A1" s="3" t="str">
+      <x:c r="A1" s="2" t="str">
         <x:v>Source Row Ledger</x:v>
       </x:c>
+      <x:c r="B1" s="2"/>
+      <x:c r="C1" s="2"/>
+      <x:c r="D1" s="2"/>
+      <x:c r="E1" s="2"/>
+      <x:c r="F1" s="2"/>
+      <x:c r="G1" s="2"/>
+      <x:c r="H1" s="2"/>
+      <x:c r="I1" s="2"/>
     </x:row>
     <x:row r="2" ht="30" customHeight="1">
-      <x:c r="A2" s="8" t="str">
+      <x:c r="A2" s="6" t="str">
         <x:v>Every source table row must appear exactly once as ACCEPTED, BLOCKED, or EXCLUDED.</x:v>
       </x:c>
+      <x:c r="B2" s="6"/>
+      <x:c r="C2" s="6"/>
+      <x:c r="D2" s="6"/>
+      <x:c r="E2" s="6"/>
+      <x:c r="F2" s="6"/>
+      <x:c r="G2" s="6"/>
+      <x:c r="H2" s="6"/>
+      <x:c r="I2" s="6"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="str">
@@ -1556,12 +1441,9 @@
     <x:mergeCell ref="A1:I1"/>
     <x:mergeCell ref="A2:I2"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="D5:F10004">
-    <x:cfRule type="containsText" dxfId="5" priority="1" operator="containsText" text="BLOCKED"/>
-  </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd5635e25ac394136"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1574,28 +1456,41 @@
     <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="14" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="14" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="20" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="18" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="55" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="60" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
-      <x:c r="A1" s="3" t="str">
+      <x:c r="A1" s="2" t="str">
         <x:v>Canonical Beam Results</x:v>
       </x:c>
-      <x:c r="E1" s="70"/>
-      <x:c r="F1" s="70"/>
-      <x:c r="G1" s="70"/>
-      <x:c r="H1" s="70"/>
-      <x:c r="I1" s="70"/>
+      <x:c r="B1" s="2"/>
+      <x:c r="C1" s="2"/>
+      <x:c r="D1" s="2"/>
+      <x:c r="E1" s="2"/>
+      <x:c r="F1" s="2"/>
+      <x:c r="G1" s="2"/>
+      <x:c r="H1" s="2"/>
+      <x:c r="I1" s="2"/>
+      <x:c r="J1" s="2"/>
     </x:row>
     <x:row r="2" ht="30" customHeight="1">
-      <x:c r="A2" s="8" t="str">
+      <x:c r="A2" s="6" t="str">
         <x:v>These are display projections of canonical-beam-result/v1. The full result envelope remains authoritative.</x:v>
       </x:c>
+      <x:c r="B2" s="6"/>
+      <x:c r="C2" s="6"/>
+      <x:c r="D2" s="6"/>
+      <x:c r="E2" s="6"/>
+      <x:c r="F2" s="6"/>
+      <x:c r="G2" s="6"/>
+      <x:c r="H2" s="6"/>
+      <x:c r="I2" s="6"/>
+      <x:c r="J2" s="6"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="str">
@@ -1646,13 +1541,9 @@
     <x:mergeCell ref="A1:J1"/>
     <x:mergeCell ref="A2:J2"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="D5:D10004">
-    <x:cfRule type="containsText" dxfId="6" priority="1" operator="containsText" text="PASS"/>
-    <x:cfRule type="containsText" dxfId="7" priority="2" operator="containsText" text="FAIL"/>
-  </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R44a0e2c3f5794949"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1664,26 +1555,48 @@
     <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="24" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="24" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="24" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="24" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="36" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="36" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="36" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="36" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="16" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="24" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="24" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="24" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="24" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="36" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="36" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="36" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="36" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
-      <x:c r="A1" s="3" t="str">
+      <x:c r="A1" s="2" t="str">
         <x:v>Calculation Passports</x:v>
       </x:c>
+      <x:c r="B1" s="2"/>
+      <x:c r="C1" s="2"/>
+      <x:c r="D1" s="2"/>
+      <x:c r="E1" s="2"/>
+      <x:c r="F1" s="2"/>
+      <x:c r="G1" s="2"/>
+      <x:c r="H1" s="2"/>
+      <x:c r="I1" s="2"/>
+      <x:c r="J1" s="2"/>
+      <x:c r="K1" s="2"/>
+      <x:c r="L1" s="2"/>
     </x:row>
     <x:row r="2" ht="30" customHeight="1">
-      <x:c r="A2" s="8" t="str">
+      <x:c r="A2" s="6" t="str">
         <x:v>Each passport binds a row, normalized input, canonical result, library content, workbook selection, and reviewed mapping.</x:v>
       </x:c>
+      <x:c r="B2" s="6"/>
+      <x:c r="C2" s="6"/>
+      <x:c r="D2" s="6"/>
+      <x:c r="E2" s="6"/>
+      <x:c r="F2" s="6"/>
+      <x:c r="G2" s="6"/>
+      <x:c r="H2" s="6"/>
+      <x:c r="I2" s="6"/>
+      <x:c r="J2" s="6"/>
+      <x:c r="K2" s="6"/>
+      <x:c r="L2" s="6"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="str">
@@ -1744,7 +1657,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdd18e0535f5d405f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>